<commit_message>
docs(spec): record Supabase preview-branch validation of security migrations
The PR's Supabase preview branch applied both new migrations cleanly (all
tasks green: Database/Migrations/Seeding/Edge Functions), confirming the SQL
the local sandbox could not execute. Update the 12 remediated rows' notes from
'pending controlled deploy' to record the preview validation; production grant
application still happens on merge/deploy.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014S52k5c2MnEwDseb6QSrmj
</commit_message>
<xml_diff>
--- a/docs/spec/2026-06-24-behavioral-spec.xlsx
+++ b/docs/spec/2026-06-24-behavioral-spec.xlsx
@@ -636,7 +636,7 @@
         <v>docs/adr/0011*.md; docs/adr/0013*.md; supabase/migrations/20260615220000_portal_ce_mercante_gate.sql</v>
       </c>
       <c r="J7" t="str">
-        <v>RESOLVED: 20260624100000_revoke_anon_portal_read_rpcs.sql revokes anon from the six Portal read RPCs; 20260624100100_guard_definer_rpcs_active_user.sql adds is_active_user() gates. Asserted by definerActiveUserGuardMigration.test.ts (green). Remote grant application pending controlled deploy.</v>
+        <v>RESOLVED: 20260624100000_revoke_anon_portal_read_rpcs.sql revokes anon from the six Portal read RPCs; 20260624100100_guard_definer_rpcs_active_user.sql adds is_active_user() gates. Asserted by definerActiveUserGuardMigration.test.ts (green). Migrations applied cleanly to the PR Supabase preview branch (all tasks green); production grant application on merge/deploy.</v>
       </c>
     </row>
     <row r="8">
@@ -2172,7 +2172,7 @@
         <v>chargeOperationsService.ts; 20260612144751_*.sql</v>
       </c>
       <c r="J55" t="str">
-        <v>RESOLVED: is_active_user() gate added in 20260624100100_guard_definer_rpcs_active_user.sql (ADR 0004); SQL readers converted to plpgsql (query preserved via RETURN QUERY). definerActiveUserGuardMigration.test.ts green. Remote grant application pending controlled deploy.</v>
+        <v>RESOLVED: is_active_user() gate added in 20260624100100_guard_definer_rpcs_active_user.sql (ADR 0004); SQL readers converted to plpgsql (query preserved via RETURN QUERY). definerActiveUserGuardMigration.test.ts green. Migrations applied cleanly to the PR Supabase preview branch (all tasks green); production grant application on merge/deploy.</v>
       </c>
     </row>
     <row r="56">
@@ -2556,7 +2556,7 @@
         <v>alerts.ts; 024_detect_overdue_invoices.sql</v>
       </c>
       <c r="J67" t="str">
-        <v>RESOLVED: is_active_user() gate added in 20260624100100_guard_definer_rpcs_active_user.sql (ADR 0004); SQL readers converted to plpgsql (query preserved via RETURN QUERY). definerActiveUserGuardMigration.test.ts green. Remote grant application pending controlled deploy.</v>
+        <v>RESOLVED: is_active_user() gate added in 20260624100100_guard_definer_rpcs_active_user.sql (ADR 0004); SQL readers converted to plpgsql (query preserved via RETURN QUERY). definerActiveUserGuardMigration.test.ts green. Migrations applied cleanly to the PR Supabase preview branch (all tasks green); production grant application on merge/deploy.</v>
       </c>
     </row>
     <row r="68">
@@ -2908,7 +2908,7 @@
         <v>chargeOperationsService.ts; 016_local_charges_stage_a.sql</v>
       </c>
       <c r="J78" t="str">
-        <v>RESOLVED: is_active_user() gate added in 20260624100100_guard_definer_rpcs_active_user.sql (ADR 0004); SQL readers converted to plpgsql (query preserved via RETURN QUERY). definerActiveUserGuardMigration.test.ts green. Remote grant application pending controlled deploy.</v>
+        <v>RESOLVED: is_active_user() gate added in 20260624100100_guard_definer_rpcs_active_user.sql (ADR 0004); SQL readers converted to plpgsql (query preserved via RETURN QUERY). definerActiveUserGuardMigration.test.ts green. Migrations applied cleanly to the PR Supabase preview branch (all tasks green); production grant application on merge/deploy.</v>
       </c>
     </row>
     <row r="79">
@@ -2972,7 +2972,7 @@
         <v>chargeReconciliationService.ts; 025_*.sql</v>
       </c>
       <c r="J80" t="str">
-        <v>RESOLVED: is_active_user() gate added in 20260624100100_guard_definer_rpcs_active_user.sql (ADR 0004); SQL readers converted to plpgsql (query preserved via RETURN QUERY). definerActiveUserGuardMigration.test.ts green. Remote grant application pending controlled deploy.</v>
+        <v>RESOLVED: is_active_user() gate added in 20260624100100_guard_definer_rpcs_active_user.sql (ADR 0004); SQL readers converted to plpgsql (query preserved via RETURN QUERY). definerActiveUserGuardMigration.test.ts green. Migrations applied cleanly to the PR Supabase preview branch (all tasks green); production grant application on merge/deploy.</v>
       </c>
     </row>
     <row r="81">
@@ -3068,7 +3068,7 @@
         <v>chargeOperationsService.ts; 019_*.sql</v>
       </c>
       <c r="J83" t="str">
-        <v>RESOLVED: is_active_user() gate added in 20260624100100_guard_definer_rpcs_active_user.sql (ADR 0004); SQL readers converted to plpgsql (query preserved via RETURN QUERY). definerActiveUserGuardMigration.test.ts green. Remote grant application pending controlled deploy.</v>
+        <v>RESOLVED: is_active_user() gate added in 20260624100100_guard_definer_rpcs_active_user.sql (ADR 0004); SQL readers converted to plpgsql (query preserved via RETURN QUERY). definerActiveUserGuardMigration.test.ts green. Migrations applied cleanly to the PR Supabase preview branch (all tasks green); production grant application on merge/deploy.</v>
       </c>
     </row>
     <row r="84">
@@ -3260,7 +3260,7 @@
         <v>portalOperation.ts; portalCeMercanteGateMigration.test.ts</v>
       </c>
       <c r="J89" t="str">
-        <v>RESOLVED: anon EXECUTE revoked in 20260624100000_revoke_anon_portal_read_rpcs.sql (ADR 0013). definerActiveUserGuardMigration.test.ts green. Remote grant application pending controlled deploy.</v>
+        <v>RESOLVED: anon EXECUTE revoked in 20260624100000_revoke_anon_portal_read_rpcs.sql (ADR 0013). definerActiveUserGuardMigration.test.ts green. Migrations applied cleanly to the PR Supabase preview branch (all tasks green); production grant application on merge/deploy.</v>
       </c>
     </row>
     <row r="90">
@@ -3900,7 +3900,7 @@
         <v>portalBilling.ts; portalInvoiceHistoryLinksMigration.test.ts</v>
       </c>
       <c r="J109" t="str">
-        <v>RESOLVED: anon EXECUTE revoked in 20260624100000_revoke_anon_portal_read_rpcs.sql (ADR 0013). definerActiveUserGuardMigration.test.ts green. Remote grant application pending controlled deploy.</v>
+        <v>RESOLVED: anon EXECUTE revoked in 20260624100000_revoke_anon_portal_read_rpcs.sql (ADR 0013). definerActiveUserGuardMigration.test.ts green. Migrations applied cleanly to the PR Supabase preview branch (all tasks green); production grant application on merge/deploy.</v>
       </c>
     </row>
     <row r="110">
@@ -3932,7 +3932,7 @@
         <v>portalBilling.ts; portalInvoiceConsolidatedBreakdownMigration.test.ts</v>
       </c>
       <c r="J110" t="str">
-        <v>RESOLVED: anon EXECUTE revoked in 20260624100000_revoke_anon_portal_read_rpcs.sql (ADR 0013). definerActiveUserGuardMigration.test.ts green. Remote grant application pending controlled deploy.</v>
+        <v>RESOLVED: anon EXECUTE revoked in 20260624100000_revoke_anon_portal_read_rpcs.sql (ADR 0013). definerActiveUserGuardMigration.test.ts green. Migrations applied cleanly to the PR Supabase preview branch (all tasks green); production grant application on merge/deploy.</v>
       </c>
     </row>
     <row r="111">
@@ -3964,7 +3964,7 @@
         <v>portalBilling.ts; portalCeMercanteGateMigration.test.ts</v>
       </c>
       <c r="J111" t="str">
-        <v>RESOLVED: anon EXECUTE revoked in 20260624100000_revoke_anon_portal_read_rpcs.sql (ADR 0013). definerActiveUserGuardMigration.test.ts green. Remote grant application pending controlled deploy.</v>
+        <v>RESOLVED: anon EXECUTE revoked in 20260624100000_revoke_anon_portal_read_rpcs.sql (ADR 0013). definerActiveUserGuardMigration.test.ts green. Migrations applied cleanly to the PR Supabase preview branch (all tasks green); production grant application on merge/deploy.</v>
       </c>
     </row>
     <row r="112">
@@ -3996,7 +3996,7 @@
         <v>portalBilling.ts; portalCeMercanteGateMigration.test.ts</v>
       </c>
       <c r="J112" t="str">
-        <v>RESOLVED: anon EXECUTE revoked in 20260624100000_revoke_anon_portal_read_rpcs.sql (ADR 0013). definerActiveUserGuardMigration.test.ts green. Remote grant application pending controlled deploy.</v>
+        <v>RESOLVED: anon EXECUTE revoked in 20260624100000_revoke_anon_portal_read_rpcs.sql (ADR 0013). definerActiveUserGuardMigration.test.ts green. Migrations applied cleanly to the PR Supabase preview branch (all tasks green); production grant application on merge/deploy.</v>
       </c>
     </row>
     <row r="113">
@@ -4028,7 +4028,7 @@
         <v>portalBilling.ts; portalCeMercanteGateMigration.test.ts</v>
       </c>
       <c r="J113" t="str">
-        <v>RESOLVED: anon EXECUTE revoked in 20260624100000_revoke_anon_portal_read_rpcs.sql (ADR 0013). definerActiveUserGuardMigration.test.ts green. Remote grant application pending controlled deploy.</v>
+        <v>RESOLVED: anon EXECUTE revoked in 20260624100000_revoke_anon_portal_read_rpcs.sql (ADR 0013). definerActiveUserGuardMigration.test.ts green. Migrations applied cleanly to the PR Supabase preview branch (all tasks green); production grant application on merge/deploy.</v>
       </c>
     </row>
     <row r="114">

</xml_diff>